<commit_message>
Update er_diargam.drawio, er_diargam.drawio.png, and normalization_task.xlsx
</commit_message>
<xml_diff>
--- a/Lab_3/normalization_task.xlsx
+++ b/Lab_3/normalization_task.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EDUCATION_2025\DEV-DB-2026. Основы БД для программистов (PostgreSQL)\DEV_DB_2026\Lab_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C383B8-76D1-4474-B37D-16BCA3548C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AEA3A0-04CB-4E47-BE53-F463819E878A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="1515" windowWidth="19275" windowHeight="18030" activeTab="3" xr2:uid="{CDDA8C1B-5D6B-4EB4-B524-45BC91F4C87D}"/>
+    <workbookView xWindow="5085" yWindow="1485" windowWidth="15420" windowHeight="18030" activeTab="4" xr2:uid="{CDDA8C1B-5D6B-4EB4-B524-45BC91F4C87D}"/>
   </bookViews>
   <sheets>
     <sheet name="Исходные данные" sheetId="1" r:id="rId1"/>
     <sheet name="1НФ" sheetId="2" r:id="rId2"/>
     <sheet name="2НФ" sheetId="3" r:id="rId3"/>
     <sheet name="3НФ" sheetId="4" r:id="rId4"/>
+    <sheet name="Схема данных" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="54">
   <si>
     <t>Код сотрудника</t>
   </si>
@@ -108,9 +109,6 @@
     <t>Linux</t>
   </si>
   <si>
-    <t>Для приведения представленной таблицы к первой нормальной форме (1НФ) необходимо устранить неатомарные значения.</t>
-  </si>
-  <si>
     <t>Что изменилось:</t>
   </si>
   <si>
@@ -144,15 +142,6 @@
     <t>2. Все неключевые атрибуты должны иметь полную функциональную зависимость от всего составного первичного ключа, а не от его части.</t>
   </si>
   <si>
-    <t>(это когда неключевой атрибут зависит от другого неключевого атрибута)</t>
-  </si>
-  <si>
-    <t>Номер отдела, в свою очередь, зависит от первичного ключа (Код сотрудника).</t>
-  </si>
-  <si>
-    <t>Проблема в текущей таблице «Сотрудники»: Наименование отдела зависит от Номера отдела.</t>
-  </si>
-  <si>
     <t>Теперь здесь хранится только информация о человеке и ссылка на его отдел.</t>
   </si>
   <si>
@@ -189,63 +178,26 @@
     <t>Чтобы достичь 3НФ, мы выносим информацию об отделах в отдельную таблицу.</t>
   </si>
   <si>
-    <t>Сотрудники -&gt; Отделы: Связь «многие к одному» (много сотрудников в одном отделе).</t>
-  </si>
-  <si>
-    <t>Сотрудники -&gt;  Квалификации: Связь «один ко многим» (у одного сотрудника много навыков).</t>
-  </si>
-  <si>
-    <r>
-      <t>Для перехода к</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0A0A0A"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t>третьей нормальной форме (3НФ) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>необходимо устранить транзитивные зависимости</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0A0A0A"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t>.</t>
-    </r>
+    <t>Для приведения представленной таблицы к первой нормальной форме (1НФ) необходимо устранить неатомарные значения (в каждой ячейке должно находиться только одно элементарное (неделимое) значение.)</t>
+  </si>
+  <si>
+    <t>Код сотрудника [PK] [FK]</t>
+  </si>
+  <si>
+    <t>В итоге:</t>
+  </si>
+  <si>
+    <t>Нет дублирования: Название «Отдел проектирования» встречается в базе только один раз.</t>
+  </si>
+  <si>
+    <t>Целостность: Мы можем создать новый отдел, даже если в нем еще нет сотрудников.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -262,20 +214,6 @@
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0A0A0A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="3">
@@ -316,14 +254,14 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -340,6 +278,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Рисунок 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAE7F035-7CA2-7D99-B2E5-2A2CB9592CB4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7324725" cy="1438275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -651,7 +644,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -671,7 +664,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="6">
+      <c r="A2" s="7">
         <v>7513</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -691,7 +684,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+      <c r="A3" s="7">
         <v>9842</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -711,7 +704,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>6651</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -731,7 +724,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+      <c r="A5" s="7">
         <v>9006</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -751,10 +744,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="A7" s="7"/>
+      <c r="B7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -776,7 +767,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -791,12 +782,12 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="6">
         <v>7513</v>
       </c>
       <c r="B2" t="s">
@@ -811,12 +802,12 @@
       <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="6">
         <v>7513</v>
       </c>
       <c r="B3" t="s">
@@ -831,12 +822,12 @@
       <c r="E3" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="6">
         <v>9842</v>
       </c>
       <c r="B4" t="s">
@@ -851,12 +842,12 @@
       <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <v>6651</v>
       </c>
       <c r="B5" t="s">
@@ -871,12 +862,12 @@
       <c r="E5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <v>6651</v>
       </c>
       <c r="B6" t="s">
@@ -891,12 +882,12 @@
       <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>9006</v>
       </c>
       <c r="B7" t="s">
@@ -911,12 +902,12 @@
       <c r="E7" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="6">
         <v>9006</v>
       </c>
       <c r="B8" t="s">
@@ -931,34 +922,34 @@
       <c r="E8" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="6"/>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -980,17 +971,17 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>45</v>
+      <c r="A3" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>1</v>
@@ -1006,7 +997,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="6">
         <v>7513</v>
       </c>
       <c r="B4" t="s">
@@ -1023,7 +1014,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <v>9842</v>
       </c>
       <c r="B5" t="s">
@@ -1040,7 +1031,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <v>6651</v>
       </c>
       <c r="B6" t="s">
@@ -1057,7 +1048,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>9006</v>
       </c>
       <c r="B7" t="s">
@@ -1075,91 +1066,91 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>50</v>
       </c>
+      <c r="B12" s="6" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <v>7513</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="6">
         <v>7513</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="6">
         <v>9842</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="6">
         <v>6651</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="A17" s="6">
         <v>6651</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+      <c r="A18" s="6">
         <v>9006</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="6">
         <v>9006</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1169,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19C10B1-4484-4F35-99F9-84D7F1C70576}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
@@ -1180,17 +1171,17 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>1</v>
@@ -1198,12 +1189,12 @@
       <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>46</v>
+      <c r="D3" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="6">
         <v>7513</v>
       </c>
       <c r="B4" t="s">
@@ -1212,12 +1203,12 @@
       <c r="C4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="6">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <v>9842</v>
       </c>
       <c r="B5" t="s">
@@ -1226,12 +1217,12 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="6">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <v>6651</v>
       </c>
       <c r="B6" t="s">
@@ -1240,12 +1231,12 @@
       <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="6">
         <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>9006</v>
       </c>
       <c r="B7" t="s">
@@ -1254,35 +1245,35 @@
       <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>47</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <v>120</v>
       </c>
       <c r="B13" t="s">
@@ -1290,7 +1281,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="6">
         <v>30</v>
       </c>
       <c r="B14" t="s">
@@ -1299,112 +1290,107 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>49</v>
+      <c r="A18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="6">
         <v>7513</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="8">
+      <c r="A20" s="6">
         <v>7513</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="A21" s="6">
         <v>9842</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="A22" s="6">
         <v>6651</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="A23" s="6">
         <v>6651</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
+      <c r="A24" s="6">
         <v>9006</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="A25" s="6">
         <v>9006</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236F5D3B-90DF-4D8A-8802-EF9A720ED2A7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>